<commit_message>
adding BINS01 in the templates
</commit_message>
<xml_diff>
--- a/000_TEMPLATE_SUBMISSION/gridConvergence_D01_V1.xlsx
+++ b/000_TEMPLATE_SUBMISSION/gridConvergence_D01_V1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mkzayni/Desktop/UNIVERSITY/IPW3/IPW3/000_TEMPLATE_SUBMISSION/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE6972EB-2B23-2D40-B880-540E0EA2315B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6365BDBA-E183-9A40-8497-F3F0481832A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17720" tabRatio="500" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INSTRUCTIONS" sheetId="1" r:id="rId1"/>
@@ -52,15 +52,6 @@
   </si>
   <si>
     <t>CMY [-]: Pitching Moment coefficient about the moment reference center (MRC)</t>
-  </si>
-  <si>
-    <t>WATER_MASS [kg]: Impinged water mass (patch or total)</t>
-  </si>
-  <si>
-    <t>ICE_MASS [kg]: Accreted Ice mass (patch or total)</t>
-  </si>
-  <si>
-    <t>WATER_EVAP_MASS [kg]: Evaporated water mass (patch or total)</t>
   </si>
   <si>
     <t xml:space="preserve"> IMPORTANT NOTES: </t>
@@ -424,6 +415,15 @@
   <si>
     <t>7-Bin KS = Variable</t>
   </si>
+  <si>
+    <t>Mass of water evaporated [kg]: Evaporated water mass (patch or total)</t>
+  </si>
+  <si>
+    <t>Mass of water impinged [kg]: Impinged water mass (patch or total)</t>
+  </si>
+  <si>
+    <t>Mass of ice accreted [kg]: Accreted Ice mass (patch or total)</t>
+  </si>
 </sst>
 </file>
 
@@ -783,6 +783,15 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -796,15 +805,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1298,22 +1298,22 @@
     </row>
     <row r="10" spans="1:1" ht="22" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
-        <v>6</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" spans="1:1" ht="22" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
-        <v>7</v>
+        <v>68</v>
       </c>
     </row>
     <row r="12" spans="1:1" ht="22" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" spans="1:1" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="54" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="16" x14ac:dyDescent="0.2">
@@ -1321,32 +1321,32 @@
     </row>
     <row r="15" spans="1:1" ht="22" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16" spans="1:1" ht="22" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="53" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -1354,60 +1354,60 @@
     </row>
     <row r="22" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E27" s="4"/>
     </row>
     <row r="28" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E30" s="4"/>
     </row>
     <row r="31" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="E31" s="4"/>
     </row>
     <row r="32" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="53" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E32" s="4"/>
     </row>
@@ -1417,66 +1417,66 @@
     </row>
     <row r="34" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E34" s="4"/>
     </row>
     <row r="35" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E35" s="4"/>
     </row>
     <row r="36" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E36" s="4"/>
     </row>
     <row r="37" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A37" s="3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E37" s="4"/>
     </row>
     <row r="38" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A38" s="3" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A39" s="3" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A40" s="3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E40" s="4"/>
     </row>
     <row r="41" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A41" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E41" s="4"/>
     </row>
     <row r="42" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A42" s="3" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E42" s="4"/>
     </row>
     <row r="43" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="E43" s="4"/>
     </row>
     <row r="44" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A44" s="53" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -1485,67 +1485,67 @@
     </row>
     <row r="46" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A46" s="3" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E46" s="4"/>
     </row>
     <row r="47" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A47" s="3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E47" s="4"/>
     </row>
     <row r="48" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A48" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E48" s="4"/>
     </row>
     <row r="49" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A49" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E49" s="4"/>
     </row>
     <row r="50" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A50" s="3" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E50" s="4"/>
     </row>
     <row r="51" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E51" s="4"/>
     </row>
     <row r="52" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A52" s="3" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E52" s="4"/>
     </row>
     <row r="53" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E53" s="4"/>
     </row>
     <row r="54" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A54" s="3" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E54" s="4"/>
     </row>
     <row r="55" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A55" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E55" s="4"/>
     </row>
     <row r="56" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A56" s="53" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -1554,37 +1554,37 @@
     </row>
     <row r="58" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E58" s="4"/>
     </row>
     <row r="59" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A59" s="5" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E59" s="4"/>
     </row>
     <row r="60" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A60" s="3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E60" s="4"/>
     </row>
     <row r="61" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E61" s="4"/>
     </row>
     <row r="62" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A62" s="3" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E62" s="4"/>
     </row>
     <row r="63" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A63" s="3" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E63" s="4"/>
     </row>
@@ -1662,75 +1662,75 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="27" x14ac:dyDescent="0.2">
-      <c r="A1" s="49" t="s">
-        <v>48</v>
-      </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
-      <c r="I1" s="49"/>
+      <c r="A1" s="52" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="52"/>
+      <c r="H1" s="52"/>
+      <c r="I1" s="52"/>
     </row>
     <row r="2" spans="1:9" ht="27" x14ac:dyDescent="0.2">
-      <c r="A2" s="50" t="s">
-        <v>60</v>
-      </c>
-      <c r="B2" s="51"/>
-      <c r="C2" s="51"/>
-      <c r="D2" s="51"/>
-      <c r="E2" s="51"/>
-      <c r="F2" s="51"/>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
-      <c r="I2" s="52"/>
+      <c r="A2" s="45" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
+      <c r="I2" s="47"/>
     </row>
     <row r="3" spans="1:9" ht="27" x14ac:dyDescent="0.2">
-      <c r="A3" s="45" t="s">
-        <v>66</v>
-      </c>
-      <c r="B3" s="45"/>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45" t="s">
-        <v>67</v>
-      </c>
-      <c r="E3" s="45"/>
-      <c r="F3" s="45"/>
-      <c r="G3" s="46" t="s">
-        <v>68</v>
-      </c>
-      <c r="H3" s="47"/>
-      <c r="I3" s="48"/>
+      <c r="A3" s="48" t="s">
+        <v>63</v>
+      </c>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48" t="s">
+        <v>64</v>
+      </c>
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="49" t="s">
+        <v>65</v>
+      </c>
+      <c r="H3" s="50"/>
+      <c r="I3" s="51"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B4" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="C4" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="D4" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E4" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="F4" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="F4" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="G4" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="H4" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I4" s="19" t="s">
         <v>55</v>
-      </c>
-      <c r="I4" s="19" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
@@ -1896,78 +1896,78 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B12" s="11"/>
       <c r="C12" s="19"/>
       <c r="D12" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E12" s="11"/>
       <c r="F12" s="19"/>
       <c r="G12" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="H12" s="11"/>
       <c r="I12" s="19"/>
     </row>
     <row r="13" spans="1:9" ht="27" x14ac:dyDescent="0.2">
-      <c r="A13" s="50" t="s">
-        <v>61</v>
-      </c>
-      <c r="B13" s="51"/>
-      <c r="C13" s="51"/>
-      <c r="D13" s="51"/>
-      <c r="E13" s="51"/>
-      <c r="F13" s="51"/>
-      <c r="G13" s="51"/>
-      <c r="H13" s="51"/>
-      <c r="I13" s="52"/>
+      <c r="A13" s="45" t="s">
+        <v>58</v>
+      </c>
+      <c r="B13" s="46"/>
+      <c r="C13" s="46"/>
+      <c r="D13" s="46"/>
+      <c r="E13" s="46"/>
+      <c r="F13" s="46"/>
+      <c r="G13" s="46"/>
+      <c r="H13" s="46"/>
+      <c r="I13" s="47"/>
     </row>
     <row r="14" spans="1:9" ht="27" x14ac:dyDescent="0.2">
-      <c r="A14" s="45" t="s">
-        <v>66</v>
-      </c>
-      <c r="B14" s="45"/>
-      <c r="C14" s="45"/>
-      <c r="D14" s="45" t="s">
-        <v>67</v>
-      </c>
-      <c r="E14" s="45"/>
-      <c r="F14" s="45"/>
-      <c r="G14" s="46" t="s">
-        <v>68</v>
-      </c>
-      <c r="H14" s="47"/>
-      <c r="I14" s="48"/>
+      <c r="A14" s="48" t="s">
+        <v>63</v>
+      </c>
+      <c r="B14" s="48"/>
+      <c r="C14" s="48"/>
+      <c r="D14" s="48" t="s">
+        <v>64</v>
+      </c>
+      <c r="E14" s="48"/>
+      <c r="F14" s="48"/>
+      <c r="G14" s="49" t="s">
+        <v>65</v>
+      </c>
+      <c r="H14" s="50"/>
+      <c r="I14" s="51"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B15" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C15" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="C15" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="D15" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E15" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="F15" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="F15" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="G15" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="H15" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I15" s="19" t="s">
         <v>55</v>
-      </c>
-      <c r="I15" s="19" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
@@ -2133,78 +2133,78 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B23" s="11"/>
       <c r="C23" s="19"/>
       <c r="D23" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E23" s="11"/>
       <c r="F23" s="19"/>
       <c r="G23" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="H23" s="11"/>
       <c r="I23" s="19"/>
     </row>
     <row r="24" spans="1:9" ht="27" x14ac:dyDescent="0.2">
-      <c r="A24" s="50" t="s">
-        <v>62</v>
-      </c>
-      <c r="B24" s="51"/>
-      <c r="C24" s="51"/>
-      <c r="D24" s="51"/>
-      <c r="E24" s="51"/>
-      <c r="F24" s="51"/>
-      <c r="G24" s="51"/>
-      <c r="H24" s="51"/>
-      <c r="I24" s="52"/>
+      <c r="A24" s="45" t="s">
+        <v>59</v>
+      </c>
+      <c r="B24" s="46"/>
+      <c r="C24" s="46"/>
+      <c r="D24" s="46"/>
+      <c r="E24" s="46"/>
+      <c r="F24" s="46"/>
+      <c r="G24" s="46"/>
+      <c r="H24" s="46"/>
+      <c r="I24" s="47"/>
     </row>
     <row r="25" spans="1:9" ht="27" x14ac:dyDescent="0.2">
-      <c r="A25" s="45" t="s">
-        <v>66</v>
-      </c>
-      <c r="B25" s="45"/>
-      <c r="C25" s="45"/>
-      <c r="D25" s="45" t="s">
-        <v>67</v>
-      </c>
-      <c r="E25" s="45"/>
-      <c r="F25" s="45"/>
-      <c r="G25" s="46" t="s">
-        <v>68</v>
-      </c>
-      <c r="H25" s="47"/>
-      <c r="I25" s="48"/>
+      <c r="A25" s="48" t="s">
+        <v>63</v>
+      </c>
+      <c r="B25" s="48"/>
+      <c r="C25" s="48"/>
+      <c r="D25" s="48" t="s">
+        <v>64</v>
+      </c>
+      <c r="E25" s="48"/>
+      <c r="F25" s="48"/>
+      <c r="G25" s="49" t="s">
+        <v>65</v>
+      </c>
+      <c r="H25" s="50"/>
+      <c r="I25" s="51"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B26" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C26" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="C26" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="D26" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E26" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="F26" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="F26" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="G26" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="H26" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I26" s="19" t="s">
         <v>55</v>
-      </c>
-      <c r="I26" s="19" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
@@ -2370,78 +2370,78 @@
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B34" s="11"/>
       <c r="C34" s="19"/>
       <c r="D34" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E34" s="11"/>
       <c r="F34" s="19"/>
       <c r="G34" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="H34" s="11"/>
       <c r="I34" s="19"/>
     </row>
     <row r="35" spans="1:9" ht="27" x14ac:dyDescent="0.2">
-      <c r="A35" s="50" t="s">
+      <c r="A35" s="45" t="s">
+        <v>60</v>
+      </c>
+      <c r="B35" s="46"/>
+      <c r="C35" s="46"/>
+      <c r="D35" s="46"/>
+      <c r="E35" s="46"/>
+      <c r="F35" s="46"/>
+      <c r="G35" s="46"/>
+      <c r="H35" s="46"/>
+      <c r="I35" s="47"/>
+    </row>
+    <row r="36" spans="1:9" ht="27" x14ac:dyDescent="0.2">
+      <c r="A36" s="48" t="s">
         <v>63</v>
       </c>
-      <c r="B35" s="51"/>
-      <c r="C35" s="51"/>
-      <c r="D35" s="51"/>
-      <c r="E35" s="51"/>
-      <c r="F35" s="51"/>
-      <c r="G35" s="51"/>
-      <c r="H35" s="51"/>
-      <c r="I35" s="52"/>
-    </row>
-    <row r="36" spans="1:9" ht="27" x14ac:dyDescent="0.2">
-      <c r="A36" s="45" t="s">
-        <v>66</v>
-      </c>
-      <c r="B36" s="45"/>
-      <c r="C36" s="45"/>
-      <c r="D36" s="45" t="s">
-        <v>67</v>
-      </c>
-      <c r="E36" s="45"/>
-      <c r="F36" s="45"/>
-      <c r="G36" s="46" t="s">
-        <v>68</v>
-      </c>
-      <c r="H36" s="47"/>
-      <c r="I36" s="48"/>
+      <c r="B36" s="48"/>
+      <c r="C36" s="48"/>
+      <c r="D36" s="48" t="s">
+        <v>64</v>
+      </c>
+      <c r="E36" s="48"/>
+      <c r="F36" s="48"/>
+      <c r="G36" s="49" t="s">
+        <v>65</v>
+      </c>
+      <c r="H36" s="50"/>
+      <c r="I36" s="51"/>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B37" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C37" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="C37" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="D37" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E37" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="F37" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="F37" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="G37" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="H37" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I37" s="19" t="s">
         <v>55</v>
-      </c>
-      <c r="I37" s="19" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.2">
@@ -2607,23 +2607,28 @@
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B45" s="11"/>
       <c r="C45" s="19"/>
       <c r="D45" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E45" s="11"/>
       <c r="F45" s="19"/>
       <c r="G45" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="H45" s="11"/>
       <c r="I45" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="D3:F3"/>
+    <mergeCell ref="G3:I3"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
     <mergeCell ref="A35:I35"/>
     <mergeCell ref="A36:C36"/>
     <mergeCell ref="D36:F36"/>
@@ -2636,11 +2641,6 @@
     <mergeCell ref="A25:C25"/>
     <mergeCell ref="D25:F25"/>
     <mergeCell ref="G25:I25"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="D3:F3"/>
-    <mergeCell ref="G3:I3"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2659,7 +2659,7 @@
   <sheetData>
     <row r="1" spans="1:1024" ht="27" x14ac:dyDescent="0.2">
       <c r="A1" s="55" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B1" s="55"/>
       <c r="C1" s="55"/>
@@ -2667,16 +2667,16 @@
     </row>
     <row r="2" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A2" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="D2" s="17" t="s">
         <v>44</v>
-      </c>
-      <c r="B2" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="C2" s="17" t="s">
-        <v>46</v>
-      </c>
-      <c r="D2" s="17" t="s">
-        <v>47</v>
       </c>
       <c r="O2" s="16"/>
       <c r="P2" s="16"/>
@@ -3713,7 +3713,7 @@
     </row>
     <row r="4" spans="1:1024" ht="27" x14ac:dyDescent="0.2">
       <c r="A4" s="55" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B4" s="55"/>
       <c r="C4" s="55"/>
@@ -3730,16 +3730,16 @@
     </row>
     <row r="5" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A5" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="D5" s="17" t="s">
         <v>44</v>
-      </c>
-      <c r="B5" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="C5" s="17" t="s">
-        <v>46</v>
-      </c>
-      <c r="D5" s="17" t="s">
-        <v>47</v>
       </c>
       <c r="G5" s="7"/>
       <c r="H5" s="7"/>
@@ -4781,7 +4781,7 @@
     </row>
     <row r="7" spans="1:1024" ht="27" x14ac:dyDescent="0.2">
       <c r="A7" s="55" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B7" s="55"/>
       <c r="C7" s="55"/>
@@ -4798,16 +4798,16 @@
     </row>
     <row r="8" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A8" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" s="17" t="s">
         <v>44</v>
-      </c>
-      <c r="B8" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="C8" s="17" t="s">
-        <v>46</v>
-      </c>
-      <c r="D8" s="17" t="s">
-        <v>47</v>
       </c>
       <c r="G8" s="7"/>
       <c r="H8" s="7"/>
@@ -5849,7 +5849,7 @@
     </row>
     <row r="10" spans="1:1024" ht="27" x14ac:dyDescent="0.2">
       <c r="A10" s="55" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B10" s="55"/>
       <c r="C10" s="55"/>
@@ -5865,16 +5865,16 @@
     </row>
     <row r="11" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A11" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="17" t="s">
         <v>44</v>
-      </c>
-      <c r="B11" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="C11" s="17" t="s">
-        <v>46</v>
-      </c>
-      <c r="D11" s="17" t="s">
-        <v>47</v>
       </c>
       <c r="J11" s="7"/>
       <c r="K11" s="7"/>
@@ -6923,7 +6923,7 @@
     </row>
     <row r="14" spans="1:1024" ht="27" x14ac:dyDescent="0.2">
       <c r="A14" s="56" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B14" s="56"/>
       <c r="C14" s="56"/>
@@ -7371,7 +7371,7 @@
   <sheetData>
     <row r="1" spans="1:18" ht="27" x14ac:dyDescent="0.2">
       <c r="A1" s="57" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B1" s="58"/>
       <c r="C1" s="58"/>
@@ -7379,16 +7379,16 @@
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" s="19" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C2" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="D2" s="19" t="s">
         <v>46</v>
-      </c>
-      <c r="D2" s="19" t="s">
-        <v>49</v>
       </c>
       <c r="E2" s="12"/>
       <c r="F2" s="12"/>
@@ -7475,7 +7475,7 @@
     </row>
     <row r="8" spans="1:18" ht="27" x14ac:dyDescent="0.2">
       <c r="A8" s="57" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B8" s="58"/>
       <c r="C8" s="58"/>
@@ -7487,16 +7487,16 @@
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" s="19" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C9" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="D9" s="19" t="s">
         <v>46</v>
-      </c>
-      <c r="D9" s="19" t="s">
-        <v>49</v>
       </c>
       <c r="E9" s="10"/>
       <c r="F9" s="10"/>
@@ -7575,7 +7575,7 @@
     </row>
     <row r="15" spans="1:18" ht="27" x14ac:dyDescent="0.2">
       <c r="A15" s="57" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B15" s="58"/>
       <c r="C15" s="58"/>
@@ -7589,16 +7589,16 @@
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A16" s="19" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C16" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="D16" s="19" t="s">
         <v>46</v>
-      </c>
-      <c r="D16" s="19" t="s">
-        <v>49</v>
       </c>
       <c r="E16" s="10"/>
       <c r="F16" s="10"/>
@@ -7691,7 +7691,7 @@
     </row>
     <row r="22" spans="1:15" ht="27" x14ac:dyDescent="0.2">
       <c r="A22" s="57" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B22" s="58"/>
       <c r="C22" s="58"/>
@@ -7705,16 +7705,16 @@
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23" s="19" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C23" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23" s="19" t="s">
         <v>46</v>
-      </c>
-      <c r="D23" s="19" t="s">
-        <v>49</v>
       </c>
       <c r="E23" s="10"/>
       <c r="F23" s="10"/>
@@ -7813,7 +7813,7 @@
     </row>
     <row r="30" spans="1:15" ht="27" x14ac:dyDescent="0.2">
       <c r="A30" s="60" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B30" s="60"/>
       <c r="C30" s="60"/>
@@ -7829,7 +7829,7 @@
     </row>
     <row r="31" spans="1:15" ht="27" x14ac:dyDescent="0.2">
       <c r="A31" s="60" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B31" s="60"/>
       <c r="C31" s="60"/>
@@ -8301,7 +8301,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="27" x14ac:dyDescent="0.2">
       <c r="A1" s="61" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B1" s="62"/>
       <c r="C1" s="62"/>
@@ -8317,87 +8317,87 @@
       <c r="M1" s="63"/>
     </row>
     <row r="2" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A2" s="45" t="s">
-        <v>60</v>
-      </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
-      <c r="M2" s="45"/>
+      <c r="A2" s="48" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
+      <c r="E2" s="48"/>
+      <c r="F2" s="48"/>
+      <c r="G2" s="48"/>
+      <c r="H2" s="48"/>
+      <c r="I2" s="48"/>
+      <c r="J2" s="48"/>
+      <c r="K2" s="48"/>
+      <c r="L2" s="48"/>
+      <c r="M2" s="48"/>
     </row>
     <row r="3" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A3" s="45" t="s">
-        <v>64</v>
-      </c>
-      <c r="B3" s="45"/>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="F3" s="45"/>
-      <c r="G3" s="45"/>
-      <c r="H3" s="46" t="s">
-        <v>52</v>
-      </c>
-      <c r="I3" s="47"/>
-      <c r="J3" s="48"/>
-      <c r="K3" s="46" t="s">
-        <v>53</v>
-      </c>
-      <c r="L3" s="47"/>
-      <c r="M3" s="48"/>
+      <c r="A3" s="48" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48"/>
+      <c r="H3" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="I3" s="50"/>
+      <c r="J3" s="51"/>
+      <c r="K3" s="49" t="s">
+        <v>50</v>
+      </c>
+      <c r="L3" s="50"/>
+      <c r="M3" s="51"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="17"/>
       <c r="B4" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="I4" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="J4" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="K4" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="L4" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M4" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B5" s="34"/>
       <c r="C5" s="34"/>
@@ -8413,87 +8413,87 @@
       <c r="M5" s="25"/>
     </row>
     <row r="6" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A6" s="50" t="s">
+      <c r="A6" s="45" t="s">
+        <v>58</v>
+      </c>
+      <c r="B6" s="46"/>
+      <c r="C6" s="46"/>
+      <c r="D6" s="46"/>
+      <c r="E6" s="46"/>
+      <c r="F6" s="46"/>
+      <c r="G6" s="46"/>
+      <c r="H6" s="46"/>
+      <c r="I6" s="46"/>
+      <c r="J6" s="46"/>
+      <c r="K6" s="46"/>
+      <c r="L6" s="46"/>
+      <c r="M6" s="47"/>
+    </row>
+    <row r="7" spans="1:13" ht="27" x14ac:dyDescent="0.2">
+      <c r="A7" s="48" t="s">
         <v>61</v>
       </c>
-      <c r="B6" s="51"/>
-      <c r="C6" s="51"/>
-      <c r="D6" s="51"/>
-      <c r="E6" s="51"/>
-      <c r="F6" s="51"/>
-      <c r="G6" s="51"/>
-      <c r="H6" s="51"/>
-      <c r="I6" s="51"/>
-      <c r="J6" s="51"/>
-      <c r="K6" s="51"/>
-      <c r="L6" s="51"/>
-      <c r="M6" s="52"/>
-    </row>
-    <row r="7" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A7" s="45" t="s">
-        <v>64</v>
-      </c>
-      <c r="B7" s="45"/>
-      <c r="C7" s="45"/>
-      <c r="D7" s="45"/>
-      <c r="E7" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="F7" s="45"/>
-      <c r="G7" s="45"/>
-      <c r="H7" s="46" t="s">
-        <v>52</v>
-      </c>
-      <c r="I7" s="47"/>
-      <c r="J7" s="48"/>
-      <c r="K7" s="46" t="s">
-        <v>53</v>
-      </c>
-      <c r="L7" s="47"/>
-      <c r="M7" s="48"/>
+      <c r="B7" s="48"/>
+      <c r="C7" s="48"/>
+      <c r="D7" s="48"/>
+      <c r="E7" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="F7" s="48"/>
+      <c r="G7" s="48"/>
+      <c r="H7" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="I7" s="50"/>
+      <c r="J7" s="51"/>
+      <c r="K7" s="49" t="s">
+        <v>50</v>
+      </c>
+      <c r="L7" s="50"/>
+      <c r="M7" s="51"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="G8" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="H8" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="I8" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="J8" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="K8" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="L8" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M8" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B9" s="34"/>
       <c r="C9" s="34"/>
@@ -8509,87 +8509,87 @@
       <c r="M9" s="25"/>
     </row>
     <row r="10" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A10" s="45" t="s">
-        <v>62</v>
-      </c>
-      <c r="B10" s="45"/>
-      <c r="C10" s="45"/>
-      <c r="D10" s="45"/>
-      <c r="E10" s="45"/>
-      <c r="F10" s="45"/>
-      <c r="G10" s="45"/>
-      <c r="H10" s="45"/>
-      <c r="I10" s="45"/>
-      <c r="J10" s="45"/>
-      <c r="K10" s="45"/>
-      <c r="L10" s="45"/>
-      <c r="M10" s="45"/>
+      <c r="A10" s="48" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" s="48"/>
+      <c r="C10" s="48"/>
+      <c r="D10" s="48"/>
+      <c r="E10" s="48"/>
+      <c r="F10" s="48"/>
+      <c r="G10" s="48"/>
+      <c r="H10" s="48"/>
+      <c r="I10" s="48"/>
+      <c r="J10" s="48"/>
+      <c r="K10" s="48"/>
+      <c r="L10" s="48"/>
+      <c r="M10" s="48"/>
     </row>
     <row r="11" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A11" s="45" t="s">
-        <v>64</v>
-      </c>
-      <c r="B11" s="45"/>
-      <c r="C11" s="45"/>
-      <c r="D11" s="45"/>
-      <c r="E11" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="F11" s="45"/>
-      <c r="G11" s="45"/>
-      <c r="H11" s="46" t="s">
-        <v>52</v>
-      </c>
-      <c r="I11" s="47"/>
-      <c r="J11" s="48"/>
-      <c r="K11" s="46" t="s">
-        <v>53</v>
-      </c>
-      <c r="L11" s="47"/>
-      <c r="M11" s="48"/>
+      <c r="A11" s="48" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" s="48"/>
+      <c r="C11" s="48"/>
+      <c r="D11" s="48"/>
+      <c r="E11" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="F11" s="48"/>
+      <c r="G11" s="48"/>
+      <c r="H11" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="I11" s="50"/>
+      <c r="J11" s="51"/>
+      <c r="K11" s="49" t="s">
+        <v>50</v>
+      </c>
+      <c r="L11" s="50"/>
+      <c r="M11" s="51"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="17"/>
       <c r="B12" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="G12" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="H12" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="I12" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="J12" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="K12" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="L12" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M12" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B13" s="34"/>
       <c r="C13" s="34"/>
@@ -8605,87 +8605,87 @@
       <c r="M13" s="41"/>
     </row>
     <row r="14" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A14" s="45" t="s">
-        <v>63</v>
-      </c>
-      <c r="B14" s="45"/>
-      <c r="C14" s="45"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="45"/>
-      <c r="F14" s="45"/>
-      <c r="G14" s="45"/>
-      <c r="H14" s="45"/>
-      <c r="I14" s="45"/>
-      <c r="J14" s="45"/>
-      <c r="K14" s="45"/>
-      <c r="L14" s="45"/>
-      <c r="M14" s="45"/>
+      <c r="A14" s="48" t="s">
+        <v>60</v>
+      </c>
+      <c r="B14" s="48"/>
+      <c r="C14" s="48"/>
+      <c r="D14" s="48"/>
+      <c r="E14" s="48"/>
+      <c r="F14" s="48"/>
+      <c r="G14" s="48"/>
+      <c r="H14" s="48"/>
+      <c r="I14" s="48"/>
+      <c r="J14" s="48"/>
+      <c r="K14" s="48"/>
+      <c r="L14" s="48"/>
+      <c r="M14" s="48"/>
     </row>
     <row r="15" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A15" s="45" t="s">
-        <v>64</v>
-      </c>
-      <c r="B15" s="45"/>
-      <c r="C15" s="45"/>
-      <c r="D15" s="45"/>
-      <c r="E15" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="F15" s="45"/>
-      <c r="G15" s="45"/>
-      <c r="H15" s="46" t="s">
-        <v>52</v>
-      </c>
-      <c r="I15" s="47"/>
-      <c r="J15" s="48"/>
-      <c r="K15" s="46" t="s">
-        <v>53</v>
-      </c>
-      <c r="L15" s="47"/>
-      <c r="M15" s="48"/>
+      <c r="A15" s="48" t="s">
+        <v>61</v>
+      </c>
+      <c r="B15" s="48"/>
+      <c r="C15" s="48"/>
+      <c r="D15" s="48"/>
+      <c r="E15" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="F15" s="48"/>
+      <c r="G15" s="48"/>
+      <c r="H15" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="I15" s="50"/>
+      <c r="J15" s="51"/>
+      <c r="K15" s="49" t="s">
+        <v>50</v>
+      </c>
+      <c r="L15" s="50"/>
+      <c r="M15" s="51"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="17"/>
       <c r="B16" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E16" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="G16" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="H16" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="I16" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="J16" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="K16" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="L16" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M16" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B17" s="34"/>
       <c r="C17" s="34"/>
@@ -8702,16 +8702,6 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="A14:M14"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="E15:G15"/>
-    <mergeCell ref="H15:J15"/>
-    <mergeCell ref="K15:M15"/>
-    <mergeCell ref="A10:M10"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="E11:G11"/>
-    <mergeCell ref="H11:J11"/>
-    <mergeCell ref="K11:M11"/>
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="K3:M3"/>
     <mergeCell ref="A2:M2"/>
@@ -8723,6 +8713,16 @@
     <mergeCell ref="E3:G3"/>
     <mergeCell ref="H3:J3"/>
     <mergeCell ref="K7:M7"/>
+    <mergeCell ref="A10:M10"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="K11:M11"/>
+    <mergeCell ref="A14:M14"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="H15:J15"/>
+    <mergeCell ref="K15:M15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -8750,58 +8750,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="27" x14ac:dyDescent="0.2">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="52" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="52"/>
+      <c r="H1" s="52"/>
+      <c r="I1" s="52"/>
+      <c r="J1" s="52"/>
+      <c r="K1" s="52"/>
+      <c r="L1" s="52"/>
+    </row>
+    <row r="2" spans="1:17" s="27" customFormat="1" ht="27" x14ac:dyDescent="0.2">
+      <c r="A2" s="48" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
+      <c r="E2" s="48"/>
+      <c r="F2" s="48"/>
+      <c r="G2" s="48"/>
+      <c r="H2" s="48"/>
+      <c r="I2" s="48"/>
+      <c r="J2" s="48"/>
+      <c r="K2" s="48"/>
+      <c r="L2" s="48"/>
+    </row>
+    <row r="3" spans="1:17" s="27" customFormat="1" ht="27" x14ac:dyDescent="0.2">
+      <c r="A3" s="48" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
-      <c r="I1" s="49"/>
-      <c r="J1" s="49"/>
-      <c r="K1" s="49"/>
-      <c r="L1" s="49"/>
-    </row>
-    <row r="2" spans="1:17" s="27" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A2" s="45" t="s">
-        <v>60</v>
-      </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
-    </row>
-    <row r="3" spans="1:17" s="27" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A3" s="45" t="s">
-        <v>64</v>
-      </c>
-      <c r="B3" s="45"/>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="E3" s="45"/>
-      <c r="F3" s="45"/>
-      <c r="G3" s="45" t="s">
-        <v>52</v>
-      </c>
-      <c r="H3" s="45"/>
-      <c r="I3" s="45"/>
-      <c r="J3" s="45" t="s">
-        <v>53</v>
-      </c>
-      <c r="K3" s="45"/>
-      <c r="L3" s="45"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48" t="s">
+        <v>49</v>
+      </c>
+      <c r="H3" s="48"/>
+      <c r="I3" s="48"/>
+      <c r="J3" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="K3" s="48"/>
+      <c r="L3" s="48"/>
       <c r="N3" s="18"/>
       <c r="O3" s="18"/>
       <c r="P3" s="18"/>
@@ -8809,40 +8809,40 @@
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A4" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B4" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="C4" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="D4" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E4" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="F4" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="F4" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="G4" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="H4" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I4" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="I4" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="J4" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K4" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="L4" s="19" t="s">
         <v>55</v>
-      </c>
-      <c r="L4" s="19" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.2">
@@ -8935,7 +8935,7 @@
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
       <c r="D8" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E8" s="42"/>
       <c r="F8" s="19"/>
@@ -9028,7 +9028,7 @@
       <c r="D12" s="10"/>
       <c r="E12" s="10"/>
       <c r="G12" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="H12" s="11"/>
       <c r="I12" s="19"/>
@@ -9177,7 +9177,7 @@
       <c r="H20" s="10"/>
       <c r="I20" s="10"/>
       <c r="J20" s="24" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="K20" s="25"/>
       <c r="L20" s="26"/>
@@ -9188,7 +9188,7 @@
     </row>
     <row r="21" spans="1:17" s="27" customFormat="1" ht="27" x14ac:dyDescent="0.2">
       <c r="A21" s="64" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B21" s="64"/>
       <c r="C21" s="64"/>
@@ -9207,66 +9207,66 @@
       <c r="Q21" s="29"/>
     </row>
     <row r="22" spans="1:17" s="27" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A22" s="45" t="s">
-        <v>64</v>
-      </c>
-      <c r="B22" s="45"/>
-      <c r="C22" s="45"/>
-      <c r="D22" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="E22" s="45"/>
-      <c r="F22" s="45"/>
-      <c r="G22" s="45" t="s">
-        <v>52</v>
-      </c>
-      <c r="H22" s="45"/>
-      <c r="I22" s="45"/>
-      <c r="J22" s="45" t="s">
-        <v>53</v>
-      </c>
-      <c r="K22" s="45"/>
-      <c r="L22" s="45"/>
+      <c r="A22" s="48" t="s">
+        <v>61</v>
+      </c>
+      <c r="B22" s="48"/>
+      <c r="C22" s="48"/>
+      <c r="D22" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="E22" s="48"/>
+      <c r="F22" s="48"/>
+      <c r="G22" s="48" t="s">
+        <v>49</v>
+      </c>
+      <c r="H22" s="48"/>
+      <c r="I22" s="48"/>
+      <c r="J22" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="K22" s="48"/>
+      <c r="L22" s="48"/>
       <c r="O22" s="29"/>
       <c r="P22" s="29"/>
       <c r="Q22" s="29"/>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A23" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B23" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C23" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="C23" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="D23" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E23" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="F23" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="F23" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="G23" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="H23" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I23" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="I23" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="J23" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K23" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="L23" s="19" t="s">
         <v>55</v>
-      </c>
-      <c r="L23" s="19" t="s">
-        <v>58</v>
       </c>
       <c r="O23" s="7"/>
       <c r="P23" s="7"/>
@@ -9359,7 +9359,7 @@
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.2">
       <c r="D27" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E27" s="11"/>
       <c r="F27" s="19"/>
@@ -9448,7 +9448,7 @@
       <c r="D31" s="10"/>
       <c r="E31" s="10"/>
       <c r="G31" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="H31" s="11"/>
       <c r="I31" s="19"/>
@@ -9589,7 +9589,7 @@
       <c r="H39" s="10"/>
       <c r="I39" s="10"/>
       <c r="J39" s="24" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="K39" s="25"/>
       <c r="L39" s="26"/>
@@ -9599,7 +9599,7 @@
     </row>
     <row r="40" spans="1:17" s="27" customFormat="1" ht="27" x14ac:dyDescent="0.2">
       <c r="A40" s="64" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B40" s="64"/>
       <c r="C40" s="64"/>
@@ -9617,63 +9617,63 @@
       <c r="Q40" s="29"/>
     </row>
     <row r="41" spans="1:17" s="27" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A41" s="45" t="s">
-        <v>64</v>
-      </c>
-      <c r="B41" s="45"/>
-      <c r="C41" s="45"/>
-      <c r="D41" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="E41" s="45"/>
-      <c r="F41" s="45"/>
-      <c r="G41" s="45" t="s">
-        <v>52</v>
-      </c>
-      <c r="H41" s="45"/>
-      <c r="I41" s="45"/>
-      <c r="J41" s="45" t="s">
-        <v>53</v>
-      </c>
-      <c r="K41" s="45"/>
-      <c r="L41" s="45"/>
+      <c r="A41" s="48" t="s">
+        <v>61</v>
+      </c>
+      <c r="B41" s="48"/>
+      <c r="C41" s="48"/>
+      <c r="D41" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="E41" s="48"/>
+      <c r="F41" s="48"/>
+      <c r="G41" s="48" t="s">
+        <v>49</v>
+      </c>
+      <c r="H41" s="48"/>
+      <c r="I41" s="48"/>
+      <c r="J41" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="K41" s="48"/>
+      <c r="L41" s="48"/>
     </row>
     <row r="42" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A42" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B42" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C42" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="C42" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="D42" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E42" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="F42" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="F42" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="G42" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="H42" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I42" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="I42" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="J42" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K42" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="L42" s="19" t="s">
         <v>55</v>
-      </c>
-      <c r="L42" s="19" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="43" spans="1:17" x14ac:dyDescent="0.2">
@@ -9754,7 +9754,7 @@
     </row>
     <row r="46" spans="1:17" x14ac:dyDescent="0.2">
       <c r="D46" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E46" s="11"/>
       <c r="F46" s="19"/>
@@ -9831,7 +9831,7 @@
       <c r="D50" s="10"/>
       <c r="E50" s="10"/>
       <c r="G50" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="H50" s="11"/>
       <c r="I50" s="19"/>
@@ -9948,85 +9948,85 @@
       <c r="H58" s="10"/>
       <c r="I58" s="10"/>
       <c r="J58" s="24" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="K58" s="25"/>
       <c r="L58" s="26"/>
     </row>
     <row r="59" spans="1:12" s="27" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A59" s="45" t="s">
-        <v>63</v>
-      </c>
-      <c r="B59" s="45"/>
-      <c r="C59" s="45"/>
-      <c r="D59" s="45"/>
-      <c r="E59" s="45"/>
-      <c r="F59" s="45"/>
-      <c r="G59" s="45"/>
-      <c r="H59" s="45"/>
-      <c r="I59" s="45"/>
-      <c r="J59" s="45"/>
-      <c r="K59" s="45"/>
-      <c r="L59" s="45"/>
+      <c r="A59" s="48" t="s">
+        <v>60</v>
+      </c>
+      <c r="B59" s="48"/>
+      <c r="C59" s="48"/>
+      <c r="D59" s="48"/>
+      <c r="E59" s="48"/>
+      <c r="F59" s="48"/>
+      <c r="G59" s="48"/>
+      <c r="H59" s="48"/>
+      <c r="I59" s="48"/>
+      <c r="J59" s="48"/>
+      <c r="K59" s="48"/>
+      <c r="L59" s="48"/>
     </row>
     <row r="60" spans="1:12" s="27" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A60" s="45" t="s">
-        <v>64</v>
-      </c>
-      <c r="B60" s="45"/>
-      <c r="C60" s="45"/>
-      <c r="D60" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="E60" s="45"/>
-      <c r="F60" s="45"/>
-      <c r="G60" s="45" t="s">
-        <v>52</v>
-      </c>
-      <c r="H60" s="45"/>
-      <c r="I60" s="45"/>
-      <c r="J60" s="45" t="s">
-        <v>53</v>
-      </c>
-      <c r="K60" s="45"/>
-      <c r="L60" s="45"/>
+      <c r="A60" s="48" t="s">
+        <v>61</v>
+      </c>
+      <c r="B60" s="48"/>
+      <c r="C60" s="48"/>
+      <c r="D60" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="E60" s="48"/>
+      <c r="F60" s="48"/>
+      <c r="G60" s="48" t="s">
+        <v>49</v>
+      </c>
+      <c r="H60" s="48"/>
+      <c r="I60" s="48"/>
+      <c r="J60" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="K60" s="48"/>
+      <c r="L60" s="48"/>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A61" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B61" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C61" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="C61" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="D61" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E61" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="F61" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="F61" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="G61" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="H61" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I61" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="I61" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="J61" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K61" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="L61" s="19" t="s">
         <v>55</v>
-      </c>
-      <c r="L61" s="19" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.2">
@@ -10107,7 +10107,7 @@
     </row>
     <row r="65" spans="4:12" x14ac:dyDescent="0.2">
       <c r="D65" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E65" s="11"/>
       <c r="F65" s="19"/>
@@ -10184,7 +10184,7 @@
       <c r="D69" s="10"/>
       <c r="E69" s="10"/>
       <c r="G69" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="H69" s="11"/>
       <c r="I69" s="19"/>
@@ -10301,18 +10301,13 @@
       <c r="H77" s="10"/>
       <c r="I77" s="10"/>
       <c r="J77" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="K77" s="11"/>
       <c r="L77" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="A60:C60"/>
-    <mergeCell ref="A40:L40"/>
-    <mergeCell ref="A59:L59"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A2:L2"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A22:C22"/>
     <mergeCell ref="A41:C41"/>
@@ -10329,6 +10324,11 @@
     <mergeCell ref="D41:F41"/>
     <mergeCell ref="G41:I41"/>
     <mergeCell ref="J41:L41"/>
+    <mergeCell ref="A60:C60"/>
+    <mergeCell ref="A40:L40"/>
+    <mergeCell ref="A59:L59"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A2:L2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -10358,7 +10358,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="27" x14ac:dyDescent="0.2">
       <c r="A1" s="61" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B1" s="62"/>
       <c r="C1" s="62"/>
@@ -10374,87 +10374,87 @@
       <c r="M1" s="63"/>
     </row>
     <row r="2" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A2" s="45" t="s">
-        <v>60</v>
-      </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
-      <c r="M2" s="45"/>
+      <c r="A2" s="48" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
+      <c r="E2" s="48"/>
+      <c r="F2" s="48"/>
+      <c r="G2" s="48"/>
+      <c r="H2" s="48"/>
+      <c r="I2" s="48"/>
+      <c r="J2" s="48"/>
+      <c r="K2" s="48"/>
+      <c r="L2" s="48"/>
+      <c r="M2" s="48"/>
     </row>
     <row r="3" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A3" s="45" t="s">
-        <v>64</v>
-      </c>
-      <c r="B3" s="45"/>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="F3" s="45"/>
-      <c r="G3" s="45"/>
-      <c r="H3" s="46" t="s">
-        <v>52</v>
-      </c>
-      <c r="I3" s="47"/>
-      <c r="J3" s="48"/>
-      <c r="K3" s="46" t="s">
-        <v>53</v>
-      </c>
-      <c r="L3" s="47"/>
-      <c r="M3" s="48"/>
+      <c r="A3" s="48" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48"/>
+      <c r="H3" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="I3" s="50"/>
+      <c r="J3" s="51"/>
+      <c r="K3" s="49" t="s">
+        <v>50</v>
+      </c>
+      <c r="L3" s="50"/>
+      <c r="M3" s="51"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="17"/>
       <c r="B4" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="I4" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="J4" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="K4" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="L4" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M4" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B5" s="34"/>
       <c r="C5" s="34"/>
@@ -10470,87 +10470,87 @@
       <c r="M5" s="34"/>
     </row>
     <row r="6" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A6" s="50" t="s">
+      <c r="A6" s="45" t="s">
+        <v>58</v>
+      </c>
+      <c r="B6" s="46"/>
+      <c r="C6" s="46"/>
+      <c r="D6" s="46"/>
+      <c r="E6" s="46"/>
+      <c r="F6" s="46"/>
+      <c r="G6" s="46"/>
+      <c r="H6" s="46"/>
+      <c r="I6" s="46"/>
+      <c r="J6" s="46"/>
+      <c r="K6" s="46"/>
+      <c r="L6" s="46"/>
+      <c r="M6" s="47"/>
+    </row>
+    <row r="7" spans="1:13" ht="27" x14ac:dyDescent="0.2">
+      <c r="A7" s="48" t="s">
         <v>61</v>
       </c>
-      <c r="B6" s="51"/>
-      <c r="C6" s="51"/>
-      <c r="D6" s="51"/>
-      <c r="E6" s="51"/>
-      <c r="F6" s="51"/>
-      <c r="G6" s="51"/>
-      <c r="H6" s="51"/>
-      <c r="I6" s="51"/>
-      <c r="J6" s="51"/>
-      <c r="K6" s="51"/>
-      <c r="L6" s="51"/>
-      <c r="M6" s="52"/>
-    </row>
-    <row r="7" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A7" s="45" t="s">
-        <v>64</v>
-      </c>
-      <c r="B7" s="45"/>
-      <c r="C7" s="45"/>
-      <c r="D7" s="45"/>
-      <c r="E7" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="F7" s="45"/>
-      <c r="G7" s="45"/>
-      <c r="H7" s="46" t="s">
-        <v>52</v>
-      </c>
-      <c r="I7" s="47"/>
-      <c r="J7" s="48"/>
-      <c r="K7" s="46" t="s">
-        <v>53</v>
-      </c>
-      <c r="L7" s="47"/>
-      <c r="M7" s="48"/>
+      <c r="B7" s="48"/>
+      <c r="C7" s="48"/>
+      <c r="D7" s="48"/>
+      <c r="E7" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="F7" s="48"/>
+      <c r="G7" s="48"/>
+      <c r="H7" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="I7" s="50"/>
+      <c r="J7" s="51"/>
+      <c r="K7" s="49" t="s">
+        <v>50</v>
+      </c>
+      <c r="L7" s="50"/>
+      <c r="M7" s="51"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="G8" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="H8" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="I8" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="J8" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="K8" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="L8" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M8" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B9" s="34"/>
       <c r="C9" s="34"/>
@@ -10566,87 +10566,87 @@
       <c r="M9" s="34"/>
     </row>
     <row r="10" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A10" s="45" t="s">
-        <v>62</v>
-      </c>
-      <c r="B10" s="45"/>
-      <c r="C10" s="45"/>
-      <c r="D10" s="45"/>
-      <c r="E10" s="45"/>
-      <c r="F10" s="45"/>
-      <c r="G10" s="45"/>
-      <c r="H10" s="45"/>
-      <c r="I10" s="45"/>
-      <c r="J10" s="45"/>
-      <c r="K10" s="45"/>
-      <c r="L10" s="45"/>
-      <c r="M10" s="45"/>
+      <c r="A10" s="48" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" s="48"/>
+      <c r="C10" s="48"/>
+      <c r="D10" s="48"/>
+      <c r="E10" s="48"/>
+      <c r="F10" s="48"/>
+      <c r="G10" s="48"/>
+      <c r="H10" s="48"/>
+      <c r="I10" s="48"/>
+      <c r="J10" s="48"/>
+      <c r="K10" s="48"/>
+      <c r="L10" s="48"/>
+      <c r="M10" s="48"/>
     </row>
     <row r="11" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A11" s="45" t="s">
-        <v>64</v>
-      </c>
-      <c r="B11" s="45"/>
-      <c r="C11" s="45"/>
-      <c r="D11" s="45"/>
-      <c r="E11" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="F11" s="45"/>
-      <c r="G11" s="45"/>
-      <c r="H11" s="46" t="s">
-        <v>52</v>
-      </c>
-      <c r="I11" s="47"/>
-      <c r="J11" s="48"/>
-      <c r="K11" s="46" t="s">
-        <v>53</v>
-      </c>
-      <c r="L11" s="47"/>
-      <c r="M11" s="48"/>
+      <c r="A11" s="48" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" s="48"/>
+      <c r="C11" s="48"/>
+      <c r="D11" s="48"/>
+      <c r="E11" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="F11" s="48"/>
+      <c r="G11" s="48"/>
+      <c r="H11" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="I11" s="50"/>
+      <c r="J11" s="51"/>
+      <c r="K11" s="49" t="s">
+        <v>50</v>
+      </c>
+      <c r="L11" s="50"/>
+      <c r="M11" s="51"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="17"/>
       <c r="B12" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="G12" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="H12" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="I12" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="J12" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="K12" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="L12" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M12" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B13" s="34"/>
       <c r="C13" s="34"/>
@@ -10662,87 +10662,87 @@
       <c r="M13" s="34"/>
     </row>
     <row r="14" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A14" s="45" t="s">
-        <v>63</v>
-      </c>
-      <c r="B14" s="45"/>
-      <c r="C14" s="45"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="45"/>
-      <c r="F14" s="45"/>
-      <c r="G14" s="45"/>
-      <c r="H14" s="45"/>
-      <c r="I14" s="45"/>
-      <c r="J14" s="45"/>
-      <c r="K14" s="45"/>
-      <c r="L14" s="45"/>
-      <c r="M14" s="45"/>
+      <c r="A14" s="48" t="s">
+        <v>60</v>
+      </c>
+      <c r="B14" s="48"/>
+      <c r="C14" s="48"/>
+      <c r="D14" s="48"/>
+      <c r="E14" s="48"/>
+      <c r="F14" s="48"/>
+      <c r="G14" s="48"/>
+      <c r="H14" s="48"/>
+      <c r="I14" s="48"/>
+      <c r="J14" s="48"/>
+      <c r="K14" s="48"/>
+      <c r="L14" s="48"/>
+      <c r="M14" s="48"/>
     </row>
     <row r="15" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A15" s="45" t="s">
-        <v>64</v>
-      </c>
-      <c r="B15" s="45"/>
-      <c r="C15" s="45"/>
-      <c r="D15" s="45"/>
-      <c r="E15" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="F15" s="45"/>
-      <c r="G15" s="45"/>
-      <c r="H15" s="46" t="s">
-        <v>52</v>
-      </c>
-      <c r="I15" s="47"/>
-      <c r="J15" s="48"/>
-      <c r="K15" s="46" t="s">
-        <v>53</v>
-      </c>
-      <c r="L15" s="47"/>
-      <c r="M15" s="48"/>
+      <c r="A15" s="48" t="s">
+        <v>61</v>
+      </c>
+      <c r="B15" s="48"/>
+      <c r="C15" s="48"/>
+      <c r="D15" s="48"/>
+      <c r="E15" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="F15" s="48"/>
+      <c r="G15" s="48"/>
+      <c r="H15" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="I15" s="50"/>
+      <c r="J15" s="51"/>
+      <c r="K15" s="49" t="s">
+        <v>50</v>
+      </c>
+      <c r="L15" s="50"/>
+      <c r="M15" s="51"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="17"/>
       <c r="B16" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E16" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="G16" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="H16" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="I16" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="J16" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="K16" s="19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="L16" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M16" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B17" s="34"/>
       <c r="C17" s="34"/>
@@ -10759,6 +10759,12 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="K3:M3"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="E15:G15"/>
     <mergeCell ref="H15:J15"/>
@@ -10774,12 +10780,6 @@
     <mergeCell ref="H11:J11"/>
     <mergeCell ref="K11:M11"/>
     <mergeCell ref="A14:M14"/>
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="E3:G3"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="K3:M3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10805,95 +10805,95 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="52" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="52"/>
+      <c r="H1" s="52"/>
+      <c r="I1" s="52"/>
+      <c r="J1" s="52"/>
+      <c r="K1" s="52"/>
+      <c r="L1" s="52"/>
+    </row>
+    <row r="2" spans="1:12" ht="27" x14ac:dyDescent="0.2">
+      <c r="A2" s="48" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
+      <c r="E2" s="48"/>
+      <c r="F2" s="48"/>
+      <c r="G2" s="48"/>
+      <c r="H2" s="48"/>
+      <c r="I2" s="48"/>
+      <c r="J2" s="48"/>
+      <c r="K2" s="48"/>
+      <c r="L2" s="48"/>
+    </row>
+    <row r="3" spans="1:12" ht="27" x14ac:dyDescent="0.2">
+      <c r="A3" s="48" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
-      <c r="I1" s="49"/>
-      <c r="J1" s="49"/>
-      <c r="K1" s="49"/>
-      <c r="L1" s="49"/>
-    </row>
-    <row r="2" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A2" s="45" t="s">
-        <v>60</v>
-      </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
-    </row>
-    <row r="3" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A3" s="45" t="s">
-        <v>64</v>
-      </c>
-      <c r="B3" s="45"/>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="E3" s="45"/>
-      <c r="F3" s="45"/>
-      <c r="G3" s="45" t="s">
-        <v>52</v>
-      </c>
-      <c r="H3" s="45"/>
-      <c r="I3" s="45"/>
-      <c r="J3" s="45" t="s">
-        <v>53</v>
-      </c>
-      <c r="K3" s="45"/>
-      <c r="L3" s="45"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48" t="s">
+        <v>49</v>
+      </c>
+      <c r="H3" s="48"/>
+      <c r="I3" s="48"/>
+      <c r="J3" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="K3" s="48"/>
+      <c r="L3" s="48"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B4" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="C4" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="D4" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E4" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="F4" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="F4" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="G4" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="H4" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I4" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="I4" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="J4" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K4" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="L4" s="19" t="s">
         <v>55</v>
-      </c>
-      <c r="L4" s="19" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
@@ -10983,7 +10983,7 @@
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
       <c r="D8" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E8" s="11"/>
       <c r="F8" s="19"/>
@@ -11076,7 +11076,7 @@
       <c r="E12" s="10"/>
       <c r="F12" s="10"/>
       <c r="G12" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="H12" s="11"/>
       <c r="I12" s="19"/>
@@ -11225,14 +11225,14 @@
       <c r="H20" s="10"/>
       <c r="I20" s="10"/>
       <c r="J20" s="24" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="K20" s="25"/>
       <c r="L20" s="26"/>
     </row>
     <row r="21" spans="1:12" ht="27" x14ac:dyDescent="0.2">
       <c r="A21" s="64" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B21" s="64"/>
       <c r="C21" s="64"/>
@@ -11247,63 +11247,63 @@
       <c r="L21" s="64"/>
     </row>
     <row r="22" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A22" s="45" t="s">
-        <v>64</v>
-      </c>
-      <c r="B22" s="45"/>
-      <c r="C22" s="45"/>
-      <c r="D22" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="E22" s="45"/>
-      <c r="F22" s="45"/>
-      <c r="G22" s="45" t="s">
-        <v>52</v>
-      </c>
-      <c r="H22" s="45"/>
-      <c r="I22" s="45"/>
-      <c r="J22" s="45" t="s">
-        <v>53</v>
-      </c>
-      <c r="K22" s="45"/>
-      <c r="L22" s="45"/>
+      <c r="A22" s="48" t="s">
+        <v>61</v>
+      </c>
+      <c r="B22" s="48"/>
+      <c r="C22" s="48"/>
+      <c r="D22" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="E22" s="48"/>
+      <c r="F22" s="48"/>
+      <c r="G22" s="48" t="s">
+        <v>49</v>
+      </c>
+      <c r="H22" s="48"/>
+      <c r="I22" s="48"/>
+      <c r="J22" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="K22" s="48"/>
+      <c r="L22" s="48"/>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B23" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C23" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="C23" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="D23" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E23" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="F23" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="F23" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="G23" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="H23" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I23" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="I23" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="J23" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K23" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="L23" s="19" t="s">
         <v>55</v>
-      </c>
-      <c r="L23" s="19" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.2">
@@ -11393,7 +11393,7 @@
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
       <c r="D27" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E27" s="11"/>
       <c r="F27" s="19"/>
@@ -11486,7 +11486,7 @@
       <c r="E31" s="10"/>
       <c r="F31" s="10"/>
       <c r="G31" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="H31" s="11"/>
       <c r="I31" s="19"/>
@@ -11635,14 +11635,14 @@
       <c r="H39" s="10"/>
       <c r="I39" s="10"/>
       <c r="J39" s="24" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="K39" s="25"/>
       <c r="L39" s="26"/>
     </row>
     <row r="40" spans="1:12" ht="27" x14ac:dyDescent="0.2">
       <c r="A40" s="64" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B40" s="64"/>
       <c r="C40" s="64"/>
@@ -11657,63 +11657,63 @@
       <c r="L40" s="64"/>
     </row>
     <row r="41" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A41" s="45" t="s">
-        <v>64</v>
-      </c>
-      <c r="B41" s="45"/>
-      <c r="C41" s="45"/>
-      <c r="D41" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="E41" s="45"/>
-      <c r="F41" s="45"/>
-      <c r="G41" s="45" t="s">
-        <v>52</v>
-      </c>
-      <c r="H41" s="45"/>
-      <c r="I41" s="45"/>
-      <c r="J41" s="45" t="s">
-        <v>53</v>
-      </c>
-      <c r="K41" s="45"/>
-      <c r="L41" s="45"/>
+      <c r="A41" s="48" t="s">
+        <v>61</v>
+      </c>
+      <c r="B41" s="48"/>
+      <c r="C41" s="48"/>
+      <c r="D41" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="E41" s="48"/>
+      <c r="F41" s="48"/>
+      <c r="G41" s="48" t="s">
+        <v>49</v>
+      </c>
+      <c r="H41" s="48"/>
+      <c r="I41" s="48"/>
+      <c r="J41" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="K41" s="48"/>
+      <c r="L41" s="48"/>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A42" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B42" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C42" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="C42" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="D42" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E42" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="F42" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="F42" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="G42" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="H42" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I42" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="I42" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="J42" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K42" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="L42" s="19" t="s">
         <v>55</v>
-      </c>
-      <c r="L42" s="19" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.2">
@@ -11803,7 +11803,7 @@
       <c r="B46" s="6"/>
       <c r="C46" s="6"/>
       <c r="D46" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E46" s="11"/>
       <c r="F46" s="19"/>
@@ -11896,7 +11896,7 @@
       <c r="E50" s="10"/>
       <c r="F50" s="10"/>
       <c r="G50" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="H50" s="11"/>
       <c r="I50" s="19"/>
@@ -12045,85 +12045,85 @@
       <c r="H58" s="10"/>
       <c r="I58" s="10"/>
       <c r="J58" s="24" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="K58" s="25"/>
       <c r="L58" s="26"/>
     </row>
     <row r="59" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A59" s="45" t="s">
-        <v>63</v>
-      </c>
-      <c r="B59" s="45"/>
-      <c r="C59" s="45"/>
-      <c r="D59" s="45"/>
-      <c r="E59" s="45"/>
-      <c r="F59" s="45"/>
-      <c r="G59" s="45"/>
-      <c r="H59" s="45"/>
-      <c r="I59" s="45"/>
-      <c r="J59" s="45"/>
-      <c r="K59" s="45"/>
-      <c r="L59" s="45"/>
+      <c r="A59" s="48" t="s">
+        <v>60</v>
+      </c>
+      <c r="B59" s="48"/>
+      <c r="C59" s="48"/>
+      <c r="D59" s="48"/>
+      <c r="E59" s="48"/>
+      <c r="F59" s="48"/>
+      <c r="G59" s="48"/>
+      <c r="H59" s="48"/>
+      <c r="I59" s="48"/>
+      <c r="J59" s="48"/>
+      <c r="K59" s="48"/>
+      <c r="L59" s="48"/>
     </row>
     <row r="60" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A60" s="45" t="s">
-        <v>64</v>
-      </c>
-      <c r="B60" s="45"/>
-      <c r="C60" s="45"/>
-      <c r="D60" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="E60" s="45"/>
-      <c r="F60" s="45"/>
-      <c r="G60" s="45" t="s">
-        <v>52</v>
-      </c>
-      <c r="H60" s="45"/>
-      <c r="I60" s="45"/>
-      <c r="J60" s="45" t="s">
-        <v>53</v>
-      </c>
-      <c r="K60" s="45"/>
-      <c r="L60" s="45"/>
+      <c r="A60" s="48" t="s">
+        <v>61</v>
+      </c>
+      <c r="B60" s="48"/>
+      <c r="C60" s="48"/>
+      <c r="D60" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="E60" s="48"/>
+      <c r="F60" s="48"/>
+      <c r="G60" s="48" t="s">
+        <v>49</v>
+      </c>
+      <c r="H60" s="48"/>
+      <c r="I60" s="48"/>
+      <c r="J60" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="K60" s="48"/>
+      <c r="L60" s="48"/>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A61" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B61" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C61" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="C61" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="D61" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E61" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="F61" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="F61" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="G61" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="H61" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I61" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="I61" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="J61" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K61" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="L61" s="19" t="s">
         <v>55</v>
-      </c>
-      <c r="L61" s="19" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.2">
@@ -12213,7 +12213,7 @@
       <c r="B65" s="6"/>
       <c r="C65" s="6"/>
       <c r="D65" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E65" s="11"/>
       <c r="F65" s="19"/>
@@ -12306,7 +12306,7 @@
       <c r="E69" s="10"/>
       <c r="F69" s="10"/>
       <c r="G69" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="H69" s="11"/>
       <c r="I69" s="19"/>
@@ -12455,13 +12455,19 @@
       <c r="H77" s="10"/>
       <c r="I77" s="10"/>
       <c r="J77" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="K77" s="11"/>
       <c r="L77" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="D3:F3"/>
+    <mergeCell ref="G3:I3"/>
+    <mergeCell ref="J3:L3"/>
     <mergeCell ref="A60:C60"/>
     <mergeCell ref="D60:F60"/>
     <mergeCell ref="G60:I60"/>
@@ -12477,12 +12483,6 @@
     <mergeCell ref="G41:I41"/>
     <mergeCell ref="J41:L41"/>
     <mergeCell ref="A59:L59"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="D3:F3"/>
-    <mergeCell ref="G3:I3"/>
-    <mergeCell ref="J3:L3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -12510,7 +12510,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="27" x14ac:dyDescent="0.2">
       <c r="A1" s="61" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B1" s="62"/>
       <c r="C1" s="62"/>
@@ -12526,87 +12526,87 @@
       <c r="M1" s="65"/>
     </row>
     <row r="2" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A2" s="46" t="s">
-        <v>60</v>
-      </c>
-      <c r="B2" s="47"/>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
-      <c r="I2" s="47"/>
-      <c r="J2" s="47"/>
-      <c r="K2" s="47"/>
-      <c r="L2" s="47"/>
-      <c r="M2" s="48"/>
+      <c r="A2" s="49" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="50"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="50"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="50"/>
+      <c r="H2" s="50"/>
+      <c r="I2" s="50"/>
+      <c r="J2" s="50"/>
+      <c r="K2" s="50"/>
+      <c r="L2" s="50"/>
+      <c r="M2" s="51"/>
     </row>
     <row r="3" spans="1:13" s="6" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A3" s="45" t="s">
-        <v>64</v>
-      </c>
-      <c r="B3" s="45"/>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="F3" s="45"/>
-      <c r="G3" s="45"/>
-      <c r="H3" s="46" t="s">
-        <v>52</v>
-      </c>
-      <c r="I3" s="47"/>
-      <c r="J3" s="48"/>
-      <c r="K3" s="46" t="s">
-        <v>53</v>
-      </c>
-      <c r="L3" s="47"/>
-      <c r="M3" s="48"/>
+      <c r="A3" s="48" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48"/>
+      <c r="H3" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="I3" s="50"/>
+      <c r="J3" s="51"/>
+      <c r="K3" s="49" t="s">
+        <v>50</v>
+      </c>
+      <c r="L3" s="50"/>
+      <c r="M3" s="51"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="38"/>
       <c r="B4" s="36" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C4" s="36" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D4" s="36" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E4" s="36" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F4" s="36" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="G4" s="36" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="H4" s="36" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="I4" s="36" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="J4" s="36" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="K4" s="36" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="L4" s="36" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M4" s="36" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="35" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B5" s="39"/>
       <c r="C5" s="39"/>
@@ -12622,87 +12622,87 @@
       <c r="M5" s="39"/>
     </row>
     <row r="6" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A6" s="46" t="s">
+      <c r="A6" s="49" t="s">
+        <v>58</v>
+      </c>
+      <c r="B6" s="50"/>
+      <c r="C6" s="50"/>
+      <c r="D6" s="50"/>
+      <c r="E6" s="50"/>
+      <c r="F6" s="50"/>
+      <c r="G6" s="50"/>
+      <c r="H6" s="50"/>
+      <c r="I6" s="50"/>
+      <c r="J6" s="50"/>
+      <c r="K6" s="50"/>
+      <c r="L6" s="50"/>
+      <c r="M6" s="51"/>
+    </row>
+    <row r="7" spans="1:13" s="6" customFormat="1" ht="27" x14ac:dyDescent="0.2">
+      <c r="A7" s="48" t="s">
         <v>61</v>
       </c>
-      <c r="B6" s="47"/>
-      <c r="C6" s="47"/>
-      <c r="D6" s="47"/>
-      <c r="E6" s="47"/>
-      <c r="F6" s="47"/>
-      <c r="G6" s="47"/>
-      <c r="H6" s="47"/>
-      <c r="I6" s="47"/>
-      <c r="J6" s="47"/>
-      <c r="K6" s="47"/>
-      <c r="L6" s="47"/>
-      <c r="M6" s="48"/>
-    </row>
-    <row r="7" spans="1:13" s="6" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A7" s="45" t="s">
-        <v>64</v>
-      </c>
-      <c r="B7" s="45"/>
-      <c r="C7" s="45"/>
-      <c r="D7" s="45"/>
-      <c r="E7" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="F7" s="45"/>
-      <c r="G7" s="45"/>
-      <c r="H7" s="46" t="s">
-        <v>52</v>
-      </c>
-      <c r="I7" s="47"/>
-      <c r="J7" s="48"/>
-      <c r="K7" s="46" t="s">
-        <v>53</v>
-      </c>
-      <c r="L7" s="47"/>
-      <c r="M7" s="48"/>
+      <c r="B7" s="48"/>
+      <c r="C7" s="48"/>
+      <c r="D7" s="48"/>
+      <c r="E7" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="F7" s="48"/>
+      <c r="G7" s="48"/>
+      <c r="H7" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="I7" s="50"/>
+      <c r="J7" s="51"/>
+      <c r="K7" s="49" t="s">
+        <v>50</v>
+      </c>
+      <c r="L7" s="50"/>
+      <c r="M7" s="51"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="38"/>
       <c r="B8" s="36" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C8" s="36" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D8" s="36" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E8" s="36" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F8" s="36" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="G8" s="36" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="H8" s="36" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="I8" s="36" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="J8" s="36" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="K8" s="36" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="L8" s="36" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M8" s="36" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="35" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B9" s="39"/>
       <c r="C9" s="39"/>
@@ -12718,87 +12718,87 @@
       <c r="M9" s="25"/>
     </row>
     <row r="10" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A10" s="46" t="s">
-        <v>62</v>
-      </c>
-      <c r="B10" s="47"/>
-      <c r="C10" s="47"/>
-      <c r="D10" s="47"/>
-      <c r="E10" s="47"/>
-      <c r="F10" s="47"/>
-      <c r="G10" s="47"/>
-      <c r="H10" s="47"/>
-      <c r="I10" s="47"/>
-      <c r="J10" s="47"/>
-      <c r="K10" s="47"/>
-      <c r="L10" s="47"/>
-      <c r="M10" s="48"/>
+      <c r="A10" s="49" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" s="50"/>
+      <c r="C10" s="50"/>
+      <c r="D10" s="50"/>
+      <c r="E10" s="50"/>
+      <c r="F10" s="50"/>
+      <c r="G10" s="50"/>
+      <c r="H10" s="50"/>
+      <c r="I10" s="50"/>
+      <c r="J10" s="50"/>
+      <c r="K10" s="50"/>
+      <c r="L10" s="50"/>
+      <c r="M10" s="51"/>
     </row>
     <row r="11" spans="1:13" s="6" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A11" s="45" t="s">
-        <v>64</v>
-      </c>
-      <c r="B11" s="45"/>
-      <c r="C11" s="45"/>
-      <c r="D11" s="45"/>
-      <c r="E11" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="F11" s="45"/>
-      <c r="G11" s="45"/>
-      <c r="H11" s="46" t="s">
-        <v>52</v>
-      </c>
-      <c r="I11" s="47"/>
-      <c r="J11" s="48"/>
-      <c r="K11" s="46" t="s">
-        <v>53</v>
-      </c>
-      <c r="L11" s="47"/>
-      <c r="M11" s="48"/>
+      <c r="A11" s="48" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" s="48"/>
+      <c r="C11" s="48"/>
+      <c r="D11" s="48"/>
+      <c r="E11" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="F11" s="48"/>
+      <c r="G11" s="48"/>
+      <c r="H11" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="I11" s="50"/>
+      <c r="J11" s="51"/>
+      <c r="K11" s="49" t="s">
+        <v>50</v>
+      </c>
+      <c r="L11" s="50"/>
+      <c r="M11" s="51"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="38"/>
       <c r="B12" s="36" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C12" s="36" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D12" s="36" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E12" s="36" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F12" s="36" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="G12" s="36" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="H12" s="36" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="I12" s="36" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="J12" s="36" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="K12" s="36" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="L12" s="36" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M12" s="36" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="35" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B13" s="39"/>
       <c r="C13" s="39"/>
@@ -12814,87 +12814,87 @@
       <c r="M13" s="41"/>
     </row>
     <row r="14" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A14" s="46" t="s">
-        <v>63</v>
-      </c>
-      <c r="B14" s="47"/>
-      <c r="C14" s="47"/>
-      <c r="D14" s="47"/>
-      <c r="E14" s="47"/>
-      <c r="F14" s="47"/>
-      <c r="G14" s="47"/>
-      <c r="H14" s="47"/>
-      <c r="I14" s="47"/>
-      <c r="J14" s="47"/>
-      <c r="K14" s="47"/>
-      <c r="L14" s="47"/>
-      <c r="M14" s="48"/>
+      <c r="A14" s="49" t="s">
+        <v>60</v>
+      </c>
+      <c r="B14" s="50"/>
+      <c r="C14" s="50"/>
+      <c r="D14" s="50"/>
+      <c r="E14" s="50"/>
+      <c r="F14" s="50"/>
+      <c r="G14" s="50"/>
+      <c r="H14" s="50"/>
+      <c r="I14" s="50"/>
+      <c r="J14" s="50"/>
+      <c r="K14" s="50"/>
+      <c r="L14" s="50"/>
+      <c r="M14" s="51"/>
     </row>
     <row r="15" spans="1:13" s="6" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A15" s="45" t="s">
-        <v>64</v>
-      </c>
-      <c r="B15" s="45"/>
-      <c r="C15" s="45"/>
-      <c r="D15" s="45"/>
-      <c r="E15" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="F15" s="45"/>
-      <c r="G15" s="45"/>
-      <c r="H15" s="46" t="s">
-        <v>52</v>
-      </c>
-      <c r="I15" s="47"/>
-      <c r="J15" s="48"/>
-      <c r="K15" s="46" t="s">
-        <v>53</v>
-      </c>
-      <c r="L15" s="47"/>
-      <c r="M15" s="48"/>
+      <c r="A15" s="48" t="s">
+        <v>61</v>
+      </c>
+      <c r="B15" s="48"/>
+      <c r="C15" s="48"/>
+      <c r="D15" s="48"/>
+      <c r="E15" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="F15" s="48"/>
+      <c r="G15" s="48"/>
+      <c r="H15" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="I15" s="50"/>
+      <c r="J15" s="51"/>
+      <c r="K15" s="49" t="s">
+        <v>50</v>
+      </c>
+      <c r="L15" s="50"/>
+      <c r="M15" s="51"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="38"/>
       <c r="B16" s="36" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C16" s="36" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D16" s="36" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E16" s="36" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="G16" s="36" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="H16" s="36" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="I16" s="36" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="J16" s="36" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="K16" s="36" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="L16" s="36" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M16" s="36" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="35" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B17" s="39"/>
       <c r="C17" s="39"/>
@@ -12911,6 +12911,12 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="K3:M3"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="E15:G15"/>
     <mergeCell ref="H15:J15"/>
@@ -12926,12 +12932,6 @@
     <mergeCell ref="H11:J11"/>
     <mergeCell ref="K11:M11"/>
     <mergeCell ref="A14:M14"/>
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="E3:G3"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="K3:M3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -12960,7 +12960,7 @@
   <sheetData>
     <row r="1" spans="1:1021" s="32" customFormat="1" ht="27" x14ac:dyDescent="0.35">
       <c r="D1" s="60" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E1" s="60"/>
       <c r="F1" s="60"/>
@@ -13981,20 +13981,20 @@
       <c r="AMG1" s="31"/>
     </row>
     <row r="2" spans="1:1021" s="32" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A2" s="45" t="s">
-        <v>60</v>
-      </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
+      <c r="A2" s="48" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
+      <c r="E2" s="48"/>
+      <c r="F2" s="48"/>
+      <c r="G2" s="48"/>
+      <c r="H2" s="48"/>
+      <c r="I2" s="48"/>
+      <c r="J2" s="48"/>
+      <c r="K2" s="48"/>
+      <c r="L2" s="48"/>
       <c r="M2" s="31"/>
       <c r="N2" s="31"/>
       <c r="O2" s="31"/>
@@ -15006,26 +15006,26 @@
       <c r="AMG2" s="31"/>
     </row>
     <row r="3" spans="1:1021" s="32" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A3" s="46" t="s">
-        <v>64</v>
-      </c>
-      <c r="B3" s="47"/>
-      <c r="C3" s="48"/>
-      <c r="D3" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="E3" s="45"/>
-      <c r="F3" s="45"/>
-      <c r="G3" s="45" t="s">
-        <v>52</v>
-      </c>
-      <c r="H3" s="45"/>
-      <c r="I3" s="45"/>
-      <c r="J3" s="45" t="s">
-        <v>53</v>
-      </c>
-      <c r="K3" s="45"/>
-      <c r="L3" s="45"/>
+      <c r="A3" s="49" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" s="50"/>
+      <c r="C3" s="51"/>
+      <c r="D3" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48" t="s">
+        <v>49</v>
+      </c>
+      <c r="H3" s="48"/>
+      <c r="I3" s="48"/>
+      <c r="J3" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="K3" s="48"/>
+      <c r="L3" s="48"/>
       <c r="M3" s="31"/>
       <c r="N3" s="31"/>
       <c r="O3" s="21"/>
@@ -16038,40 +16038,40 @@
     </row>
     <row r="4" spans="1:1021" x14ac:dyDescent="0.2">
       <c r="A4" s="35" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B4" s="36" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" s="36" t="s">
         <v>55</v>
       </c>
-      <c r="C4" s="36" t="s">
-        <v>58</v>
-      </c>
       <c r="D4" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E4" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="F4" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="F4" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="G4" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="H4" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I4" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="I4" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="J4" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K4" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="L4" s="19" t="s">
         <v>55</v>
-      </c>
-      <c r="L4" s="19" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:1021" x14ac:dyDescent="0.2">
@@ -16152,7 +16152,7 @@
     </row>
     <row r="8" spans="1:1021" x14ac:dyDescent="0.2">
       <c r="D8" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E8" s="11"/>
       <c r="F8" s="19"/>
@@ -16221,7 +16221,7 @@
     </row>
     <row r="12" spans="1:1021" x14ac:dyDescent="0.2">
       <c r="G12" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="H12" s="42"/>
       <c r="I12" s="19"/>
@@ -16298,7 +16298,7 @@
     </row>
     <row r="20" spans="1:1021" x14ac:dyDescent="0.2">
       <c r="J20" s="24" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="K20" s="44"/>
       <c r="L20" s="24"/>
@@ -16306,20 +16306,20 @@
       <c r="N20" s="15"/>
     </row>
     <row r="21" spans="1:1021" s="32" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A21" s="45" t="s">
-        <v>61</v>
-      </c>
-      <c r="B21" s="45"/>
-      <c r="C21" s="45"/>
-      <c r="D21" s="45"/>
-      <c r="E21" s="45"/>
-      <c r="F21" s="45"/>
-      <c r="G21" s="45"/>
-      <c r="H21" s="45"/>
-      <c r="I21" s="45"/>
-      <c r="J21" s="45"/>
-      <c r="K21" s="45"/>
-      <c r="L21" s="45"/>
+      <c r="A21" s="48" t="s">
+        <v>58</v>
+      </c>
+      <c r="B21" s="48"/>
+      <c r="C21" s="48"/>
+      <c r="D21" s="48"/>
+      <c r="E21" s="48"/>
+      <c r="F21" s="48"/>
+      <c r="G21" s="48"/>
+      <c r="H21" s="48"/>
+      <c r="I21" s="48"/>
+      <c r="J21" s="48"/>
+      <c r="K21" s="48"/>
+      <c r="L21" s="48"/>
       <c r="M21" s="33"/>
       <c r="N21" s="33"/>
       <c r="O21" s="31"/>
@@ -17331,26 +17331,26 @@
       <c r="AMG21" s="31"/>
     </row>
     <row r="22" spans="1:1021" s="32" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A22" s="46" t="s">
-        <v>64</v>
-      </c>
-      <c r="B22" s="47"/>
-      <c r="C22" s="48"/>
-      <c r="D22" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="E22" s="45"/>
-      <c r="F22" s="45"/>
-      <c r="G22" s="45" t="s">
-        <v>52</v>
-      </c>
-      <c r="H22" s="45"/>
-      <c r="I22" s="45"/>
-      <c r="J22" s="45" t="s">
-        <v>53</v>
-      </c>
-      <c r="K22" s="45"/>
-      <c r="L22" s="45"/>
+      <c r="A22" s="49" t="s">
+        <v>61</v>
+      </c>
+      <c r="B22" s="50"/>
+      <c r="C22" s="51"/>
+      <c r="D22" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="E22" s="48"/>
+      <c r="F22" s="48"/>
+      <c r="G22" s="48" t="s">
+        <v>49</v>
+      </c>
+      <c r="H22" s="48"/>
+      <c r="I22" s="48"/>
+      <c r="J22" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="K22" s="48"/>
+      <c r="L22" s="48"/>
       <c r="M22" s="31"/>
       <c r="N22" s="31"/>
       <c r="O22" s="31"/>
@@ -18363,40 +18363,40 @@
     </row>
     <row r="23" spans="1:1021" x14ac:dyDescent="0.2">
       <c r="A23" s="35" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B23" s="36" t="s">
+        <v>52</v>
+      </c>
+      <c r="C23" s="36" t="s">
         <v>55</v>
       </c>
-      <c r="C23" s="36" t="s">
-        <v>58</v>
-      </c>
       <c r="D23" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E23" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="F23" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="F23" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="G23" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="H23" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I23" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="I23" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="J23" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K23" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="L23" s="19" t="s">
         <v>55</v>
-      </c>
-      <c r="L23" s="19" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="24" spans="1:1021" x14ac:dyDescent="0.2">
@@ -18477,7 +18477,7 @@
     </row>
     <row r="27" spans="1:1021" x14ac:dyDescent="0.2">
       <c r="D27" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E27" s="11"/>
       <c r="F27" s="19"/>
@@ -18546,7 +18546,7 @@
     </row>
     <row r="31" spans="1:1021" x14ac:dyDescent="0.2">
       <c r="G31" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="H31" s="42"/>
       <c r="I31" s="19"/>
@@ -18623,14 +18623,14 @@
     </row>
     <row r="39" spans="1:1021" x14ac:dyDescent="0.2">
       <c r="J39" s="24" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="K39" s="44"/>
       <c r="L39" s="24"/>
     </row>
     <row r="40" spans="1:1021" s="32" customFormat="1" ht="27" x14ac:dyDescent="0.35">
       <c r="A40" s="64" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B40" s="64"/>
       <c r="C40" s="64"/>
@@ -19654,26 +19654,26 @@
       <c r="AMG40" s="31"/>
     </row>
     <row r="41" spans="1:1021" s="32" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A41" s="46" t="s">
-        <v>64</v>
-      </c>
-      <c r="B41" s="47"/>
-      <c r="C41" s="48"/>
-      <c r="D41" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="E41" s="45"/>
-      <c r="F41" s="45"/>
-      <c r="G41" s="45" t="s">
-        <v>52</v>
-      </c>
-      <c r="H41" s="45"/>
-      <c r="I41" s="45"/>
-      <c r="J41" s="45" t="s">
-        <v>53</v>
-      </c>
-      <c r="K41" s="45"/>
-      <c r="L41" s="45"/>
+      <c r="A41" s="49" t="s">
+        <v>61</v>
+      </c>
+      <c r="B41" s="50"/>
+      <c r="C41" s="51"/>
+      <c r="D41" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="E41" s="48"/>
+      <c r="F41" s="48"/>
+      <c r="G41" s="48" t="s">
+        <v>49</v>
+      </c>
+      <c r="H41" s="48"/>
+      <c r="I41" s="48"/>
+      <c r="J41" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="K41" s="48"/>
+      <c r="L41" s="48"/>
       <c r="M41" s="31"/>
       <c r="N41" s="31"/>
       <c r="O41" s="31"/>
@@ -20686,40 +20686,40 @@
     </row>
     <row r="42" spans="1:1021" x14ac:dyDescent="0.2">
       <c r="A42" s="35" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B42" s="36" t="s">
+        <v>52</v>
+      </c>
+      <c r="C42" s="36" t="s">
         <v>55</v>
       </c>
-      <c r="C42" s="36" t="s">
-        <v>58</v>
-      </c>
       <c r="D42" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E42" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="F42" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="F42" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="G42" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="H42" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I42" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="I42" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="J42" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K42" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="L42" s="19" t="s">
         <v>55</v>
-      </c>
-      <c r="L42" s="19" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="43" spans="1:1021" x14ac:dyDescent="0.2">
@@ -20800,7 +20800,7 @@
     </row>
     <row r="46" spans="1:1021" x14ac:dyDescent="0.2">
       <c r="D46" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E46" s="11"/>
       <c r="F46" s="19"/>
@@ -20869,7 +20869,7 @@
     </row>
     <row r="50" spans="1:1021" x14ac:dyDescent="0.2">
       <c r="G50" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="H50" s="11"/>
       <c r="I50" s="19"/>
@@ -20946,14 +20946,14 @@
     </row>
     <row r="58" spans="1:1021" x14ac:dyDescent="0.2">
       <c r="J58" s="24" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="K58" s="25"/>
       <c r="L58" s="24"/>
     </row>
     <row r="59" spans="1:1021" s="32" customFormat="1" ht="27" x14ac:dyDescent="0.35">
       <c r="A59" s="64" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B59" s="64"/>
       <c r="C59" s="64"/>
@@ -21977,26 +21977,26 @@
       <c r="AMG59" s="31"/>
     </row>
     <row r="60" spans="1:1021" s="32" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A60" s="46" t="s">
-        <v>64</v>
-      </c>
-      <c r="B60" s="47"/>
-      <c r="C60" s="48"/>
-      <c r="D60" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="E60" s="45"/>
-      <c r="F60" s="45"/>
-      <c r="G60" s="45" t="s">
-        <v>52</v>
-      </c>
-      <c r="H60" s="45"/>
-      <c r="I60" s="45"/>
-      <c r="J60" s="45" t="s">
-        <v>53</v>
-      </c>
-      <c r="K60" s="45"/>
-      <c r="L60" s="45"/>
+      <c r="A60" s="49" t="s">
+        <v>61</v>
+      </c>
+      <c r="B60" s="50"/>
+      <c r="C60" s="51"/>
+      <c r="D60" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="E60" s="48"/>
+      <c r="F60" s="48"/>
+      <c r="G60" s="48" t="s">
+        <v>49</v>
+      </c>
+      <c r="H60" s="48"/>
+      <c r="I60" s="48"/>
+      <c r="J60" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="K60" s="48"/>
+      <c r="L60" s="48"/>
       <c r="M60" s="31"/>
       <c r="N60" s="31"/>
       <c r="O60" s="31"/>
@@ -23009,40 +23009,40 @@
     </row>
     <row r="61" spans="1:1021" x14ac:dyDescent="0.2">
       <c r="A61" s="35" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B61" s="36" t="s">
+        <v>52</v>
+      </c>
+      <c r="C61" s="36" t="s">
         <v>55</v>
       </c>
-      <c r="C61" s="36" t="s">
-        <v>58</v>
-      </c>
       <c r="D61" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E61" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="F61" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="F61" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="G61" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="H61" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I61" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="I61" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="J61" s="19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K61" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="L61" s="19" t="s">
         <v>55</v>
-      </c>
-      <c r="L61" s="19" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="62" spans="1:1021" x14ac:dyDescent="0.2">
@@ -23121,7 +23121,7 @@
     </row>
     <row r="65" spans="4:12" x14ac:dyDescent="0.2">
       <c r="D65" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E65" s="11"/>
       <c r="F65" s="19"/>
@@ -23190,7 +23190,7 @@
     </row>
     <row r="69" spans="4:12" x14ac:dyDescent="0.2">
       <c r="G69" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="H69" s="11"/>
       <c r="I69" s="19"/>
@@ -23267,13 +23267,21 @@
     </row>
     <row r="77" spans="4:12" x14ac:dyDescent="0.2">
       <c r="J77" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="K77" s="11"/>
       <c r="L77" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="D1:L1"/>
+    <mergeCell ref="J41:L41"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="G22:I22"/>
+    <mergeCell ref="J22:L22"/>
+    <mergeCell ref="D3:F3"/>
+    <mergeCell ref="G3:I3"/>
+    <mergeCell ref="J3:L3"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A22:C22"/>
     <mergeCell ref="A41:C41"/>
@@ -23287,14 +23295,6 @@
     <mergeCell ref="J60:L60"/>
     <mergeCell ref="D41:F41"/>
     <mergeCell ref="G41:I41"/>
-    <mergeCell ref="D1:L1"/>
-    <mergeCell ref="J41:L41"/>
-    <mergeCell ref="D22:F22"/>
-    <mergeCell ref="G22:I22"/>
-    <mergeCell ref="J22:L22"/>
-    <mergeCell ref="D3:F3"/>
-    <mergeCell ref="G3:I3"/>
-    <mergeCell ref="J3:L3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>